<commit_message>
Updating API Error Consolidated list
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1D7F6CC-54AD-42C7-B0CB-9E02EA1564DF}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F27C65BC-D0D9-433E-BB92-6B3979DEC4EF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="4" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="2" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -39,28 +39,17 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'International Prices'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">Tracking!$A$1:$G$6</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4212" uniqueCount="1049">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="1066">
   <si>
     <t>API</t>
   </si>
@@ -3238,6 +3227,57 @@
   </si>
   <si>
     <t>only non-profit rate indicators 'PN' and 'NN' are allowed when nonProfit is true</t>
+  </si>
+  <si>
+    <t>ADVISORY - currently {X}% of serial numbers in trackingNUmber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period.</t>
+  </si>
+  <si>
+    <t>WARNING - currently {X}% of serial numbers in trackingNUmber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period. COnsider updating LABEL_OWNER role MID within the Payment Authorization token or updating packageDescription.serialNumberFormat to EXTENDED to increase serial number range</t>
+  </si>
+  <si>
+    <t>CRITICAL - Currently {X}% of serial numbers in trackingNumber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period. at 100% label generation on {mid-stc-channel-source} will be bocked. Update LABEL_OWNER role MID within the Payment Authorization token or update packageDescription.serialNumberFormat to EXTENDED to avoid issues</t>
+  </si>
+  <si>
+    <t>Could not find available serial in range. All serials are currently in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source}. Update LABEL_OWNER role MID within the Payment Authorization token or update packageDescription.serialNumberFormat to EXTENDED to continue generating labels.</t>
+  </si>
+  <si>
+    <t>IMpb</t>
+  </si>
+  <si>
+    <t>https://apis.usps.com/labels/v3/</t>
+  </si>
+  <si>
+    <t>DANGEROUS_GOODS is not a supported contentType for customsForm</t>
+  </si>
+  <si>
+    <t>mailClass &lt;mailClass&gt; is not available to &lt;destinationEntryFacilityType&gt;</t>
+  </si>
+  <si>
+    <t>mailClass PARCEL_SELECT requires a destinationEntryFacilityType</t>
+  </si>
+  <si>
+    <t>originFacility and bypassFacility cannot be used at the same time</t>
+  </si>
+  <si>
+    <t>bypassFacility is only valid for GroundAdvantage/Priority Mail Containers</t>
+  </si>
+  <si>
+    <t>originFacility is only valid for GroundAdvantage/Priority Mail Containers</t>
+  </si>
+  <si>
+    <t>originFacility, bypassFacility</t>
+  </si>
+  <si>
+    <t>bypassFacility</t>
+  </si>
+  <si>
+    <t>originFacility</t>
+  </si>
+  <si>
+    <t>DestinationEntryFacilityType</t>
+  </si>
+  <si>
+    <t>destinationEntryFacilityAddress must not be populated when destinationEntryFacilityType is NONE</t>
   </si>
 </sst>
 </file>
@@ -3542,9 +3582,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3582,7 +3622,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3688,7 +3728,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3830,7 +3870,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -7819,7 +7859,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -7827,7 +7867,7 @@
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="66.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="99.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8220,6 +8260,121 @@
       </c>
       <c r="G17" s="2" t="s">
         <v>1012</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="10">
+        <v>401</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="E18" s="17">
+        <v>160427</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="10">
+        <v>402</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="E19" s="17">
+        <v>160428</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="10">
+        <v>403</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="E20" s="17">
+        <v>160430</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>1061</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="10">
+        <v>404</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="E21" s="17">
+        <v>160431</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>1062</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="10">
+        <v>405</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="E22" s="17">
+        <v>160432</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>1063</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>1060</v>
       </c>
     </row>
   </sheetData>
@@ -8232,7 +8387,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G241"/>
+  <dimension ref="A1:H247"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13754,7 +13909,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="241" spans="1:7">
+    <row r="241" spans="1:8">
       <c r="A241" s="20" t="s">
         <v>87</v>
       </c>
@@ -13776,6 +13931,145 @@
       <c r="G241" s="2" t="s">
         <v>1048</v>
       </c>
+    </row>
+    <row r="242" spans="1:8" ht="30">
+      <c r="A242" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B242" s="20">
+        <v>400</v>
+      </c>
+      <c r="C242" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D242" s="21" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E242" s="17">
+        <v>160423</v>
+      </c>
+      <c r="F242" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G242" s="2" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="243" spans="1:8" ht="45">
+      <c r="A243" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B243" s="20">
+        <v>400</v>
+      </c>
+      <c r="C243" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D243" s="21" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E243" s="17">
+        <v>160424</v>
+      </c>
+      <c r="F243" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G243" s="2" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="244" spans="1:8" ht="60">
+      <c r="A244" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B244" s="20">
+        <v>400</v>
+      </c>
+      <c r="C244" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D244" s="21" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E244" s="17">
+        <v>160425</v>
+      </c>
+      <c r="F244" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G244" s="2" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="245" spans="1:8" ht="45">
+      <c r="A245" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B245" s="20">
+        <v>400</v>
+      </c>
+      <c r="C245" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D245" s="21" t="s">
+        <v>1054</v>
+      </c>
+      <c r="E245" s="17">
+        <v>160426</v>
+      </c>
+      <c r="F245" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G245" s="2" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="246" spans="1:8">
+      <c r="A246" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B246" s="20">
+        <v>400</v>
+      </c>
+      <c r="C246" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D246" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E246" s="17">
+        <v>160429</v>
+      </c>
+      <c r="F246" t="s">
+        <v>763</v>
+      </c>
+      <c r="G246" s="2" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="247" spans="1:8">
+      <c r="A247" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B247" s="20">
+        <v>401</v>
+      </c>
+      <c r="C247" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D247" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E247" s="17">
+        <v>160433</v>
+      </c>
+      <c r="F247" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G247" s="2" t="s">
+        <v>1065</v>
+      </c>
+      <c r="H247" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{A36F69E6-5AC8-443F-8567-4E3FB7E927F1}"/>
@@ -13790,7 +14084,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G193"/>
+  <dimension ref="A1:G198"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -18198,6 +18492,121 @@
       </c>
       <c r="G193" s="2" t="s">
         <v>1011</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" ht="30">
+      <c r="A194" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B194" s="21">
+        <v>400</v>
+      </c>
+      <c r="C194" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D194" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="E194" s="17">
+        <v>160423</v>
+      </c>
+      <c r="F194" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G194" s="2" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" ht="60">
+      <c r="A195" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B195" s="21">
+        <v>400</v>
+      </c>
+      <c r="C195" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D195" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="E195" s="17">
+        <v>160424</v>
+      </c>
+      <c r="F195" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G195" s="2" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" ht="60">
+      <c r="A196" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B196" s="21">
+        <v>400</v>
+      </c>
+      <c r="C196" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D196" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="E196" s="17">
+        <v>160425</v>
+      </c>
+      <c r="F196" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G196" s="2" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" ht="45">
+      <c r="A197" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B197" s="21">
+        <v>400</v>
+      </c>
+      <c r="C197" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D197" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="E197" s="17">
+        <v>160426</v>
+      </c>
+      <c r="F197" t="s">
+        <v>1053</v>
+      </c>
+      <c r="G197" s="2" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7">
+      <c r="A198" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B198" s="21">
+        <v>400</v>
+      </c>
+      <c r="C198" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D198" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="E198" s="17">
+        <v>160429</v>
+      </c>
+      <c r="F198" t="s">
+        <v>763</v>
+      </c>
+      <c r="G198" s="2" t="s">
+        <v>1055</v>
       </c>
     </row>
   </sheetData>
@@ -19314,7 +19723,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -20306,6 +20715,38 @@
       <c r="G43" s="2" t="s">
         <v>1016</v>
       </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
+        <v>475</v>
+      </c>
+      <c r="B44">
+        <v>401</v>
+      </c>
+      <c r="C44" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" t="s">
+        <v>969</v>
+      </c>
+      <c r="E44" s="17">
+        <v>160429</v>
+      </c>
+      <c r="F44" t="s">
+        <v>763</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="E45" s="17"/>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="E46" s="17"/>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="E47" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21219,19 +21660,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -21477,6 +21905,19 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
   <ds:schemaRefs>
@@ -21486,24 +21927,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21523,6 +21946,24 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6c9b68e5-0371-4f27-93af-8d15f794dc29}" enabled="1" method="Privileged" siteId="{a01f407a-85cb-4a16-98bb-f28e6384bd28}" removed="0"/>

</xml_diff>

<commit_message>
Error List Update 9-24-2026
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D0716CE-67CE-4B6F-B395-5995874699B3}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9EBBC50E-230F-4F01-84B8-9B9B43575592}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="2" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="4" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4292" uniqueCount="1064">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4262" uniqueCount="1061">
   <si>
     <t>API</t>
   </si>
@@ -3227,15 +3227,6 @@
   </si>
   <si>
     <t>only non-profit rate indicators 'PN' and 'NN' are allowed when nonProfit is true</t>
-  </si>
-  <si>
-    <t>ADVISORY - currently {X}% of serial numbers in trackingNUmber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period.</t>
-  </si>
-  <si>
-    <t>WARNING - currently {X}% of serial numbers in trackingNUmber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period. COnsider updating LABEL_OWNER role MID within the Payment Authorization token or updating packageDescription.serialNumberFormat to EXTENDED to increase serial number range</t>
-  </si>
-  <si>
-    <t>CRITICAL - Currently {X}% of serial numbers in trackingNumber range are in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source} for 120 day period. at 100% label generation on {mid-stc-channel-source} will be bocked. Update LABEL_OWNER role MID within the Payment Authorization token or update packageDescription.serialNumberFormat to EXTENDED to avoid issues</t>
   </si>
   <si>
     <t>Could not find available serial in range. All serials are currently in use for MID {mid}, STC {stc}, Channel {channel}, and Source {source}. Update LABEL_OWNER role MID within the Payment Authorization token or update packageDescription.serialNumberFormat to EXTENDED to continue generating labels.</t>
@@ -3415,7 +3406,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3556,6 +3547,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -4721,7 +4715,7 @@
         <v>882</v>
       </c>
       <c r="B20" s="10">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>18</v>
@@ -7853,7 +7847,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -8261,7 +8255,7 @@
         <v>68</v>
       </c>
       <c r="B18" s="10">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>18</v>
@@ -8276,7 +8270,7 @@
         <v>807</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8284,7 +8278,7 @@
         <v>68</v>
       </c>
       <c r="B19" s="10">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>18</v>
@@ -8299,7 +8293,7 @@
         <v>807</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -8307,7 +8301,7 @@
         <v>68</v>
       </c>
       <c r="B20" s="10">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>18</v>
@@ -8319,10 +8313,10 @@
         <v>160430</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>1061</v>
+        <v>1058</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>1058</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -8330,7 +8324,7 @@
         <v>68</v>
       </c>
       <c r="B21" s="10">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="C21" s="10" t="s">
         <v>18</v>
@@ -8342,10 +8336,10 @@
         <v>160431</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>1062</v>
+        <v>1059</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>1059</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -8353,7 +8347,7 @@
         <v>68</v>
       </c>
       <c r="B22" s="10">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>18</v>
@@ -8365,11 +8359,20 @@
         <v>160432</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>1060</v>
-      </c>
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="E23" s="50"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="E24" s="50"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="E25" s="50"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8381,7 +8384,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:H247"/>
+  <dimension ref="A1:H244"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13926,7 +13929,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="242" spans="1:8" ht="30">
+    <row r="242" spans="1:8" ht="45">
       <c r="A242" s="20" t="s">
         <v>87</v>
       </c>
@@ -13937,19 +13940,19 @@
         <v>18</v>
       </c>
       <c r="D242" s="21" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="E242" s="17">
-        <v>160423</v>
+        <v>160426</v>
       </c>
       <c r="F242" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="G242" s="2" t="s">
         <v>1049</v>
       </c>
     </row>
-    <row r="243" spans="1:8" ht="45">
+    <row r="243" spans="1:8">
       <c r="A243" s="20" t="s">
         <v>87</v>
       </c>
@@ -13960,96 +13963,27 @@
         <v>18</v>
       </c>
       <c r="D243" s="21" t="s">
-        <v>1054</v>
+        <v>958</v>
       </c>
       <c r="E243" s="17">
-        <v>160424</v>
+        <v>160429</v>
       </c>
       <c r="F243" t="s">
-        <v>1053</v>
+        <v>763</v>
       </c>
       <c r="G243" s="2" t="s">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="244" spans="1:8" ht="60">
-      <c r="A244" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B244" s="20">
-        <v>400</v>
-      </c>
-      <c r="C244" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D244" s="21" t="s">
-        <v>1054</v>
-      </c>
-      <c r="E244" s="17">
-        <v>160425</v>
-      </c>
-      <c r="F244" t="s">
-        <v>1053</v>
-      </c>
-      <c r="G244" s="2" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="245" spans="1:8" ht="45">
-      <c r="A245" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B245" s="20">
-        <v>400</v>
-      </c>
-      <c r="C245" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D245" s="21" t="s">
-        <v>1054</v>
-      </c>
-      <c r="E245" s="17">
-        <v>160426</v>
-      </c>
-      <c r="F245" t="s">
-        <v>1053</v>
-      </c>
-      <c r="G245" s="2" t="s">
         <v>1052</v>
       </c>
     </row>
-    <row r="246" spans="1:8">
-      <c r="A246" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="B246" s="20">
-        <v>400</v>
-      </c>
-      <c r="C246" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D246" s="21" t="s">
-        <v>958</v>
-      </c>
-      <c r="E246" s="17">
-        <v>160429</v>
-      </c>
-      <c r="F246" t="s">
-        <v>763</v>
-      </c>
-      <c r="G246" s="2" t="s">
-        <v>1055</v>
-      </c>
-    </row>
-    <row r="247" spans="1:8">
-      <c r="A247" s="20"/>
-      <c r="B247" s="20"/>
-      <c r="C247" s="20"/>
-      <c r="D247" s="21"/>
-      <c r="E247" s="17"/>
-      <c r="F247"/>
-      <c r="G247" s="2"/>
-      <c r="H247" s="17"/>
+    <row r="244" spans="1:8">
+      <c r="A244" s="20"/>
+      <c r="B244" s="20"/>
+      <c r="C244" s="20"/>
+      <c r="D244" s="21"/>
+      <c r="E244" s="17"/>
+      <c r="F244"/>
+      <c r="G244" s="2"/>
+      <c r="H244" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{A36F69E6-5AC8-443F-8567-4E3FB7E927F1}"/>
@@ -14064,7 +13998,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G198"/>
+  <dimension ref="A1:G195"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -18474,7 +18408,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="194" spans="1:7" ht="30">
+    <row r="194" spans="1:7" ht="45">
       <c r="A194" s="10" t="s">
         <v>369</v>
       </c>
@@ -18488,16 +18422,16 @@
         <v>964</v>
       </c>
       <c r="E194" s="17">
-        <v>160423</v>
+        <v>160426</v>
       </c>
       <c r="F194" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="G194" s="2" t="s">
         <v>1049</v>
       </c>
     </row>
-    <row r="195" spans="1:7" ht="60">
+    <row r="195" spans="1:7">
       <c r="A195" s="10" t="s">
         <v>369</v>
       </c>
@@ -18511,82 +18445,13 @@
         <v>964</v>
       </c>
       <c r="E195" s="17">
-        <v>160424</v>
+        <v>160429</v>
       </c>
       <c r="F195" t="s">
-        <v>1053</v>
+        <v>763</v>
       </c>
       <c r="G195" s="2" t="s">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7" ht="60">
-      <c r="A196" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="B196" s="21">
-        <v>400</v>
-      </c>
-      <c r="C196" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="D196" s="10" t="s">
-        <v>964</v>
-      </c>
-      <c r="E196" s="17">
-        <v>160425</v>
-      </c>
-      <c r="F196" t="s">
-        <v>1053</v>
-      </c>
-      <c r="G196" s="2" t="s">
-        <v>1051</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7" ht="45">
-      <c r="A197" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="B197" s="21">
-        <v>400</v>
-      </c>
-      <c r="C197" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="D197" s="10" t="s">
-        <v>964</v>
-      </c>
-      <c r="E197" s="17">
-        <v>160426</v>
-      </c>
-      <c r="F197" t="s">
-        <v>1053</v>
-      </c>
-      <c r="G197" s="2" t="s">
         <v>1052</v>
-      </c>
-    </row>
-    <row r="198" spans="1:7">
-      <c r="A198" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="B198" s="21">
-        <v>400</v>
-      </c>
-      <c r="C198" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="D198" s="10" t="s">
-        <v>964</v>
-      </c>
-      <c r="E198" s="17">
-        <v>160429</v>
-      </c>
-      <c r="F198" t="s">
-        <v>763</v>
-      </c>
-      <c r="G198" s="2" t="s">
-        <v>1055</v>
       </c>
     </row>
   </sheetData>
@@ -20701,7 +20566,7 @@
         <v>475</v>
       </c>
       <c r="B44">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C44" t="s">
         <v>18</v>
@@ -20716,7 +20581,7 @@
         <v>763</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="45" spans="1:7">

</xml_diff>

<commit_message>
Updates for Error list 10/29/2026
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9EBBC50E-230F-4F01-84B8-9B9B43575592}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A441410-63E4-4737-81C6-5B4BD93A7FFF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="4" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4262" uniqueCount="1061">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4316" uniqueCount="1078">
   <si>
     <t>API</t>
   </si>
@@ -3263,6 +3263,57 @@
   </si>
   <si>
     <t>originFacility</t>
+  </si>
+  <si>
+    <t>idempotency key</t>
+  </si>
+  <si>
+    <t>This scan form can no longer be regenerated because it was created more than 30 calendar days ago.</t>
+  </si>
+  <si>
+    <t>The request payload does not match the payload saved for this X-Idempotency-Key.</t>
+  </si>
+  <si>
+    <t>customsForm.incoterm</t>
+  </si>
+  <si>
+    <t>InternationalPackageRequest.customsForm.europeanUnionProductID</t>
+  </si>
+  <si>
+    <t>InternationalPackageRequest.packageDescription.dutiesTaxesFeesPaidSeparately</t>
+  </si>
+  <si>
+    <t>InternationalPackageRequest.customsForm.DDPServiceProvider</t>
+  </si>
+  <si>
+    <t>InternationalPackageRequest.customsForm.destinationCurrencyConversionRate</t>
+  </si>
+  <si>
+    <t>InternationalPackageRequest.customsForm.destinationCurrency</t>
+  </si>
+  <si>
+    <t>incoterm is required when providing europeanUnionProductID values</t>
+  </si>
+  <si>
+    <t>customsForm.europeanUnionProductID values of merchantProductIdentifier and nonstandardizedManufacturerProductIdentifier are required when shipping [customsContentType] to [destinationCountry]</t>
+  </si>
+  <si>
+    <t>when incoterm is provided and europeanUnionProductID.merchantProductIdentifier is provided, then europeanUnionProductID.nonstandardizedManufacturerProductIdentifier must also be provided</t>
+  </si>
+  <si>
+    <t>DDPServiceProvider is not valid</t>
+  </si>
+  <si>
+    <t>destinationCurrency must contain exactly three uppercase letters</t>
+  </si>
+  <si>
+    <t>destinationCurrencyConversionRate must be a finite number from 0.00001 through 9999999.99999</t>
+  </si>
+  <si>
+    <t>codeAmountDueSender</t>
+  </si>
+  <si>
+    <t>extraService 915 or 917 is required with codAmountDueSender</t>
   </si>
 </sst>
 </file>
@@ -5362,7 +5413,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
@@ -5784,6 +5835,52 @@
       </c>
       <c r="G18" s="2" t="s">
         <v>1007</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="10" t="s">
+        <v>572</v>
+      </c>
+      <c r="B19" s="10">
+        <v>400</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="E19" s="24">
+        <v>160436</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>1061</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="10" t="s">
+        <v>572</v>
+      </c>
+      <c r="B20" s="10">
+        <v>400</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="E20" s="24">
+        <v>160437</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>1061</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>1063</v>
       </c>
     </row>
   </sheetData>
@@ -13976,13 +14073,27 @@
       </c>
     </row>
     <row r="244" spans="1:8">
-      <c r="A244" s="20"/>
-      <c r="B244" s="20"/>
-      <c r="C244" s="20"/>
-      <c r="D244" s="21"/>
-      <c r="E244" s="17"/>
-      <c r="F244"/>
-      <c r="G244" s="2"/>
+      <c r="A244" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B244" s="20">
+        <v>400</v>
+      </c>
+      <c r="C244" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D244" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E244" s="17">
+        <v>160438</v>
+      </c>
+      <c r="F244" t="s">
+        <v>1076</v>
+      </c>
+      <c r="G244" s="2" t="s">
+        <v>1077</v>
+      </c>
       <c r="H244" s="17"/>
     </row>
   </sheetData>
@@ -19568,7 +19679,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -20577,7 +20688,7 @@
       <c r="E44" s="17">
         <v>160429</v>
       </c>
-      <c r="F44" t="s">
+      <c r="F44" s="24" t="s">
         <v>763</v>
       </c>
       <c r="G44" s="2" t="s">
@@ -20585,13 +20696,186 @@
       </c>
     </row>
     <row r="45" spans="1:7">
-      <c r="E45" s="17"/>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="E46" s="17"/>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="E47" s="17"/>
+      <c r="A45" t="s">
+        <v>475</v>
+      </c>
+      <c r="B45">
+        <v>400</v>
+      </c>
+      <c r="C45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" t="s">
+        <v>969</v>
+      </c>
+      <c r="E45" s="17">
+        <v>160439</v>
+      </c>
+      <c r="F45" s="24" t="s">
+        <v>1064</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="45">
+      <c r="A46" t="s">
+        <v>475</v>
+      </c>
+      <c r="B46">
+        <v>400</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" t="s">
+        <v>969</v>
+      </c>
+      <c r="E46" s="17">
+        <v>160440</v>
+      </c>
+      <c r="F46" s="24" t="s">
+        <v>1065</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="45">
+      <c r="A47" t="s">
+        <v>475</v>
+      </c>
+      <c r="B47">
+        <v>400</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" t="s">
+        <v>969</v>
+      </c>
+      <c r="E47" s="17">
+        <v>160441</v>
+      </c>
+      <c r="F47" s="24" t="s">
+        <v>1065</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" t="s">
+        <v>475</v>
+      </c>
+      <c r="B48">
+        <v>400</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" t="s">
+        <v>969</v>
+      </c>
+      <c r="E48" s="17">
+        <v>160442</v>
+      </c>
+      <c r="F48" s="24" t="s">
+        <v>1066</v>
+      </c>
+      <c r="G48" s="2"/>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" t="s">
+        <v>475</v>
+      </c>
+      <c r="B49">
+        <v>400</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" t="s">
+        <v>969</v>
+      </c>
+      <c r="E49" s="17">
+        <v>160443</v>
+      </c>
+      <c r="F49" s="24" t="s">
+        <v>1067</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
+        <v>475</v>
+      </c>
+      <c r="B50">
+        <v>400</v>
+      </c>
+      <c r="C50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" t="s">
+        <v>969</v>
+      </c>
+      <c r="E50" s="17">
+        <v>160444</v>
+      </c>
+      <c r="F50" s="24" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" t="s">
+        <v>475</v>
+      </c>
+      <c r="B51">
+        <v>400</v>
+      </c>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" t="s">
+        <v>969</v>
+      </c>
+      <c r="E51" s="17">
+        <v>160445</v>
+      </c>
+      <c r="F51" s="24" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" t="s">
+        <v>475</v>
+      </c>
+      <c r="B52">
+        <v>400</v>
+      </c>
+      <c r="C52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" t="s">
+        <v>969</v>
+      </c>
+      <c r="E52" s="17">
+        <v>160446</v>
+      </c>
+      <c r="F52" s="24" t="s">
+        <v>1069</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>1075</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21496,6 +21780,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -21741,15 +22034,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -21764,6 +22048,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21779,14 +22071,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>